<commit_message>
feat: add support for English report generation alongside Arabic
- Introduced `build_report_en.py` to generate English Word documents from translated JSON.
- Updated `generate_word_report` to handle both Arabic and English reports, saving them with appropriate suffixes.
- Enhanced `RealAnalyzer` to produce English report JSON and updated relevant functions to manage English document paths.
- Added translation functionality for Arabic report JSON to English using a dedicated LLM.
- Included a new logo asset for report cover pages.

This commit enhances the reporting capabilities by providing bilingual support, improving accessibility for English-speaking users.
</commit_message>
<xml_diff>
--- a/real/inquiries-output/Fujairah_Police_Inquiry_Triage_Detail.xlsx
+++ b/real/inquiries-output/Fujairah_Police_Inquiry_Triage_Detail.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>تاريخ التقرير: 2026-05-09</t>
+          <t>تاريخ التقرير: 2026-05-12</t>
         </is>
       </c>
     </row>
@@ -974,12 +974,12 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>شكوى على خطأ تقني أو في النظام</t>
+          <t>شكوى عن عدم استلام الخدمة</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>العميل دفع مبلغاً لطلب PCC لكن التطبيق يظهر الدفع ملغى مما يشير إلى خطأ تقني في النظام، وهذا فشل في الخدمة يستحق تصنيفاً كشكوى على الخطأ التقني.</t>
+          <t>العميل دفع مبلغ المال للحصول على شهادة البطاقة الرمادية (PCC) لكن الخدمة لم يتم استلامها، والنظام يظهر الدفع كملغى. هذه حالة فشل في الخدمة مع خسارة مالية.</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>العميل يؤكد أن المخالفة المرورية خاطئة والصورة المرفقة ليست لدراجته ولم يكن في الفجيرة قط، وهذا اعتراض على مخالفة مشكوك فيها.</t>
+          <t>العميل يشتكي من مخالفة مرورية غير صحيحة باسمه والصورة لا تتطابق مع دراجته النارية، وطلب إزالة المخالفة. الحل الإجرائي يؤكد وجود خطأ يتطلب تصحيح.</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>المتعاملة تقدم شكراً وثناءً صريحاً على الخدمة الممتازة والتعاون والأخلاق والمعاملة الطيبة من فريق مركز الشرطة وتحديداً لعبد الله وأمل والنقيب يوسف.</t>
+          <t>العميلة تقدم شكراً وثناءً واضحاً لمركز شرطة التحريات على الخدمة الممتازة والمعاملة الحسنة في قضيتها، وتشيد بأداء الموظفين بالاسم.</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>العميل اشترى رقمين من الفجيرة وأحدهما ظهر في التطبيق والآخر لم يظهر، وقد أكدت الرسالة وجود عطل في النظام تم حله من قبلهم.</t>
+          <t>العميل اشترى رقمي تسجيل للمركبات وأحدهما لم ينزل في التطبيق. الحل أكد وجود عطل في النظام، مما يؤكد أن هذه حالة خطأ تقني.</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>العميل أكمل الفحص الدوري للمخدرات وفقاً للنظام لكن موظفو الفحص غيروا شيئاً في النظام وأعادوا إطالة الفحص، وهذا خطأ تقني أو إجرائي.</t>
+          <t>العميل يشتكي من أن النظام تم تغييره بشكل خاطئ حيث أظهر أن الفحص الدوري مكتمل لكن تم تمديد المدة 9 أشهر إضافية بدون سبب واضح.</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>العميل يقدم شكوى جادة بشأن عدم وجود حواجز خرسانية في مناطق شمالية بها وديان عميقة مما أدى لحادث وفاة، وينتقد عدم اهتمام شرطة المرور بتتبع أثر الحوادث.</t>
+          <t>العميل يشتكي من غياب الحواجز الخرسانية في المناطق الشمالية التي أدت لسقوط سيارات في الوديان وحدوث وفيات، ويشتكي أيضاً من عدم اهتمام المرور بتتبع أسباب الحوادث.</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>العميل يواجه مشكلة عند التنازل عن لوحة مميزة وخدمة العملاء طلبت منه تقديم شكوى، والرسالة تؤكد وجود عطل سابق في النظام.</t>
+          <t>العميل يواجه مشكلة في تنازله عن لوحة مميزة والحل أكد وجود عطل سابق في النظام، مما يشير إلى خطأ تقني يؤثر على معاملته.</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>العميل تلقى مخالفة على رقم سيارة ليس باسمه والرقم بدون كود، مما منعه من تجديد السيارة، وحاول التواصل مع المرور لكن لم يحصل على رد.</t>
+          <t>العميل تلقى مخالفة على رقم سيارة ليس باسمه والرقم بدون كود صحيح، ويواجه عدم القدرة على تجديد السيارة. الحل أكد عطلاً في النظام يتطلب معالجة.</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>العميل يقدم اعتراضاً صريحاً على مخالفات مرورية متعددة ويشرح ظروفه الشخصية ويطلب تخفيضها لأن المبلغ كبير جداً بالنسبة لراتبه.</t>
+          <t>العميل يعترض على عدة مخالفات مسجلة باسمه ويطلب تخفيفها بسبب الظروف الطارئة. الحل يشير إلى عطل في النظام تم اكتشافه.</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1848,12 +1848,12 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>شكوى على خطأ تقني أو في النظام</t>
+          <t>شكوى عن عدم استلام الخدمة</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>العميل دفع مبلغاً لطلب PCC لكن التطبيق يظهر الدفع ملغى مما يشير إلى خطأ تقني في النظام، وهذا فشل في الخدمة يستحق تصنيفاً كشكوى على الخطأ التقني.</t>
+          <t>العميل دفع مبلغ المال للحصول على شهادة البطاقة الرمادية (PCC) لكن الخدمة لم يتم استلامها، والنظام يظهر الدفع كملغى. هذه حالة فشل في الخدمة مع خسارة مالية.</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>العميل يؤكد أن المخالفة المرورية خاطئة والصورة المرفقة ليست لدراجته ولم يكن في الفجيرة قط، وهذا اعتراض على مخالفة مشكوك فيها.</t>
+          <t>العميل يشتكي من مخالفة مرورية غير صحيحة باسمه والصورة لا تتطابق مع دراجته النارية، وطلب إزالة المخالفة. الحل الإجرائي يؤكد وجود خطأ يتطلب تصحيح.</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
@@ -1993,7 +1993,7 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>العميل اشترى رقمين من الفجيرة وأحدهما ظهر في التطبيق والآخر لم يظهر، وقد أكدت الرسالة وجود عطل في النظام تم حله من قبلهم.</t>
+          <t>العميل اشترى رقمي تسجيل للمركبات وأحدهما لم ينزل في التطبيق. الحل أكد وجود عطل في النظام، مما يؤكد أن هذه حالة خطأ تقني.</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>العميل أكمل الفحص الدوري للمخدرات وفقاً للنظام لكن موظفو الفحص غيروا شيئاً في النظام وأعادوا إطالة الفحص، وهذا خطأ تقني أو إجرائي.</t>
+          <t>العميل يشتكي من أن النظام تم تغييره بشكل خاطئ حيث أظهر أن الفحص الدوري مكتمل لكن تم تمديد المدة 9 أشهر إضافية بدون سبب واضح.</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
@@ -2136,7 +2136,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>العميل يقدم شكوى جادة بشأن عدم وجود حواجز خرسانية في مناطق شمالية بها وديان عميقة مما أدى لحادث وفاة، وينتقد عدم اهتمام شرطة المرور بتتبع أثر الحوادث.</t>
+          <t>العميل يشتكي من غياب الحواجز الخرسانية في المناطق الشمالية التي أدت لسقوط سيارات في الوديان وحدوث وفيات، ويشتكي أيضاً من عدم اهتمام المرور بتتبع أسباب الحوادث.</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>العميل يواجه مشكلة عند التنازل عن لوحة مميزة وخدمة العملاء طلبت منه تقديم شكوى، والرسالة تؤكد وجود عطل سابق في النظام.</t>
+          <t>العميل يواجه مشكلة في تنازله عن لوحة مميزة والحل أكد وجود عطل سابق في النظام، مما يشير إلى خطأ تقني يؤثر على معاملته.</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>العميل تلقى مخالفة على رقم سيارة ليس باسمه والرقم بدون كود، مما منعه من تجديد السيارة، وحاول التواصل مع المرور لكن لم يحصل على رد.</t>
+          <t>العميل تلقى مخالفة على رقم سيارة ليس باسمه والرقم بدون كود صحيح، ويواجه عدم القدرة على تجديد السيارة. الحل أكد عطلاً في النظام يتطلب معالجة.</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>العميل يقدم اعتراضاً صريحاً على مخالفات مرورية متعددة ويشرح ظروفه الشخصية ويطلب تخفيضها لأن المبلغ كبير جداً بالنسبة لراتبه.</t>
+          <t>العميل يعترض على عدة مخالفات مسجلة باسمه ويطلب تخفيفها بسبب الظروف الطارئة. الحل يشير إلى عطل في النظام تم اكتشافه.</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>المتعاملة تقدم شكراً وثناءً صريحاً على الخدمة الممتازة والتعاون والأخلاق والمعاملة الطيبة من فريق مركز الشرطة وتحديداً لعبد الله وأمل والنقيب يوسف.</t>
+          <t>العميلة تقدم شكراً وثناءً واضحاً لمركز شرطة التحريات على الخدمة الممتازة والمعاملة الحسنة في قضيتها، وتشيد بأداء الموظفين بالاسم.</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -3032,12 +3032,12 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>شكوى على خطأ تقني أو في النظام</t>
+          <t>شكوى عن عدم استلام الخدمة</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>العميل دفع مبلغاً لطلب PCC لكن التطبيق يظهر الدفع ملغى مما يشير إلى خطأ تقني في النظام، وهذا فشل في الخدمة يستحق تصنيفاً كشكوى على الخطأ التقني.</t>
+          <t>العميل دفع مبلغ المال للحصول على شهادة البطاقة الرمادية (PCC) لكن الخدمة لم يتم استلامها، والنظام يظهر الدفع كملغى. هذه حالة فشل في الخدمة مع خسارة مالية.</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>العميل يؤكد أن المخالفة المرورية خاطئة والصورة المرفقة ليست لدراجته ولم يكن في الفجيرة قط، وهذا اعتراض على مخالفة مشكوك فيها.</t>
+          <t>العميل يشتكي من مخالفة مرورية غير صحيحة باسمه والصورة لا تتطابق مع دراجته النارية، وطلب إزالة المخالفة. الحل الإجرائي يؤكد وجود خطأ يتطلب تصحيح.</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
@@ -3172,7 +3172,7 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>المتعاملة تقدم شكراً وثناءً صريحاً على الخدمة الممتازة والتعاون والأخلاق والمعاملة الطيبة من فريق مركز الشرطة وتحديداً لعبد الله وأمل والنقيب يوسف.</t>
+          <t>العميلة تقدم شكراً وثناءً واضحاً لمركز شرطة التحريات على الخدمة الممتازة والمعاملة الحسنة في قضيتها، وتشيد بأداء الموظفين بالاسم.</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -3243,7 +3243,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>العميل اشترى رقمين من الفجيرة وأحدهما ظهر في التطبيق والآخر لم يظهر، وقد أكدت الرسالة وجود عطل في النظام تم حله من قبلهم.</t>
+          <t>العميل اشترى رقمي تسجيل للمركبات وأحدهما لم ينزل في التطبيق. الحل أكد وجود عطل في النظام، مما يؤكد أن هذه حالة خطأ تقني.</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
@@ -3311,7 +3311,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>العميل أكمل الفحص الدوري للمخدرات وفقاً للنظام لكن موظفو الفحص غيروا شيئاً في النظام وأعادوا إطالة الفحص، وهذا خطأ تقني أو إجرائي.</t>
+          <t>العميل يشتكي من أن النظام تم تغييره بشكل خاطئ حيث أظهر أن الفحص الدوري مكتمل لكن تم تمديد المدة 9 أشهر إضافية بدون سبب واضح.</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>العميل يقدم شكوى جادة بشأن عدم وجود حواجز خرسانية في مناطق شمالية بها وديان عميقة مما أدى لحادث وفاة، وينتقد عدم اهتمام شرطة المرور بتتبع أثر الحوادث.</t>
+          <t>العميل يشتكي من غياب الحواجز الخرسانية في المناطق الشمالية التي أدت لسقوط سيارات في الوديان وحدوث وفيات، ويشتكي أيضاً من عدم اهتمام المرور بتتبع أسباب الحوادث.</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
@@ -3459,7 +3459,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>العميل يواجه مشكلة عند التنازل عن لوحة مميزة وخدمة العملاء طلبت منه تقديم شكوى، والرسالة تؤكد وجود عطل سابق في النظام.</t>
+          <t>العميل يواجه مشكلة في تنازله عن لوحة مميزة والحل أكد وجود عطل سابق في النظام، مما يشير إلى خطأ تقني يؤثر على معاملته.</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -3527,7 +3527,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>العميل تلقى مخالفة على رقم سيارة ليس باسمه والرقم بدون كود، مما منعه من تجديد السيارة، وحاول التواصل مع المرور لكن لم يحصل على رد.</t>
+          <t>العميل تلقى مخالفة على رقم سيارة ليس باسمه والرقم بدون كود صحيح، ويواجه عدم القدرة على تجديد السيارة. الحل أكد عطلاً في النظام يتطلب معالجة.</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>العميل يقدم اعتراضاً صريحاً على مخالفات مرورية متعددة ويشرح ظروفه الشخصية ويطلب تخفيضها لأن المبلغ كبير جداً بالنسبة لراتبه.</t>
+          <t>العميل يعترض على عدة مخالفات مسجلة باسمه ويطلب تخفيفها بسبب الظروف الطارئة. الحل يشير إلى عطل في النظام تم اكتشافه.</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">

</xml_diff>